<commit_message>
WRite the code in optimizer.py for assigning the hours to the professors. At this point there is no optimization, we are just looking for a possible solution. In control.py I create a parallel function for checking that the solution satisfy all the constrains. In main.py all the files are called in order to load the data, find a solution and check that the solution is acceptable.
</commit_message>
<xml_diff>
--- a/data/school_schedule.xlsx
+++ b/data/school_schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Matias\Documents\ProjectosRandom\school_schedule\school_schedule\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C50A6D32-FB1D-4D2B-A908-FD5C4A5224D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFCF0C83-07AD-4D57-9491-21CFD8E2EA8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="12" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1690,7 +1690,8 @@
   <dimension ref="A1:U9"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="16" width="5.21875" customWidth="1"/>
+    <col min="2" max="10" width="9.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="16" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>